<commit_message>
vault backup: 2026-07-05 08:22:38
</commit_message>
<xml_diff>
--- a/second_brain/09_Exports/Dproperty_OS_Financial_Model.xlsx
+++ b/second_brain/09_Exports/Dproperty_OS_Financial_Model.xlsx
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -134,6 +134,8 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B26"/>
+  <dimension ref="B1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -519,14 +521,14 @@
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>Version: v0.6 (working)   Last built: 2026-07-04   Owner: Esteban</t>
+          <t>Version: v0.7 (working)   Last built: 2026-07-05   Owner: Esteban</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Basis: collected-GCI royalty, 30k/40k staged launch fee, Dproperty Select fixed pct of sale price.</t>
+          <t>Basis: collected-GCI royalty on GROSS-INTO-COMPANY, 30k/40k staged launch fee, Dproperty Select fixed pct of sale price.</t>
         </is>
       </c>
     </row>
@@ -534,92 +536,92 @@
       <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>HOW TO USE</t>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>COMMISSION WATERFALL (local franchise sale)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>1. Edit only the yellow cells on 'Assumptions' and the yellow cost rows on 'Model'.</t>
+          <t>5% commission charged -&gt; 50/50 with external advisors -&gt; 2.5% enters company.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>2. Everything else on 'Model' is a live formula and recalculates when you open in Excel.</t>
+          <t>Of what enters: 35% seller, 10% sales director, 55% franchise net.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>3. Blue rows = section headers. Grey rows = totals.</t>
+          <t>Royalty (6%) + Network &amp; Brand Fund (1.5%) are charged on GROSS-INTO-COMPANY (the 2.5%),</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>NOT on franchise net - so a franchise cannot lower royalty by inflating agent pay.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>WHAT THIS MODEL IS / IS NOT</t>
-        </is>
-      </c>
+      <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>- A transparent, adjustable operating model for the conservative 5-year plan (5 branded / 20 white-label / 15 developer).</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>HOW TO USE</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>- NOT audited. Cost lines are planning estimates. Confirm with owners before pitch-final use.</t>
+          <t>1. Edit only the yellow cells on 'Assumptions' and the yellow cost rows on 'Model'.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2. Everything else on 'Model' is a live formula and recalculates when you open in Excel.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>KEY LEVERS (Assumptions sheet)</t>
+          <t>3. Blue rows = section headers. Grey rows = totals.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>- local_comm_rate: set to 0.0075 to run the 0.75pct deferred-advisory sensitivity.</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>- select_mix / local_mix: share of a franchise's volume that is Dproperty Select vs local.</t>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>WHAT THIS MODEL IS / IS NOT</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>- ramp row (Model row 12): how fast new franchises reach full productivity.</t>
+          <t>- A transparent, adjustable operating model for the conservative 5-year plan (5 branded / 20 white-label / 15 developer).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>- dev_rev_per_project: conservative 40k blended assumption.</t>
+          <t>- NOT audited. Cost lines are planning estimates. Confirm with owners before pitch-final use.</t>
         </is>
       </c>
     </row>
@@ -629,42 +631,73 @@
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>OPEN VALIDATION ITEMS (mirror Business Plan Section 19)</t>
+          <t>KEY LEVERS (Assumptions sheet)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>1. Commission rate 5pct vs 0.75pct (Fernando/Ernesto) - BLOCKS everything.</t>
+          <t>- local_comm_rate: set to 0.0075 to run the 0.75pct deferred-advisory sensitivity.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>2. Miguel salary amount (EUR 3,000/mo placeholder).</t>
+          <t>- external_advisor_share: 0.50 = 50/50 co-broke. Set 0 for deals with no external advisor.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>3. Sales mix 70/30, ramp curve, developer per project.</t>
+          <t>- select_mix / local_mix: share of a franchise's volume that is Dproperty Select vs local.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
+          <t>- ramp row (Model row 12): how fast new franchises reach full productivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>OPEN VALIDATION ITEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1. Owner-validate the OPEX/staffing rows (drives EBITDA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2. Miguel salary amount (EUR 3,000/mo placeholder).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>3. Sales mix 70/30, ramp curve, developer per project, external-advisor share.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
           <t>4. Minimum royalty floor amount (750/mo placeholder).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>5. Whether franchisee pays royalty on Dproperty Select earnings (default: no).</t>
         </is>
       </c>
     </row>
@@ -679,13 +712,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D25"/>
+  <dimension ref="B1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -738,7 +771,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>On collected local GCI</t>
+          <t>On gross-into-company</t>
         </is>
       </c>
     </row>
@@ -753,7 +786,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>On collected local GCI</t>
+          <t>On gross-into-company</t>
         </is>
       </c>
     </row>
@@ -1001,46 +1034,139 @@
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>GCI per unit</t>
-        </is>
-      </c>
-      <c r="C23" s="11">
-        <f>C3*C4</f>
-        <v/>
+          <t>External advisor share</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Price x commission</t>
+          <t>Co-broke split; company keeps the rest</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>Select HQ retained - branded</t>
+          <t>Gross commission / unit (5pct)</t>
         </is>
       </c>
       <c r="C24" s="11">
-        <f>C3*C4-C3*C13</f>
+        <f>C3*C4</f>
         <v/>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Commission minus branded payout</t>
+          <t>Price x commission</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
+          <t>Commission into company / unit</t>
+        </is>
+      </c>
+      <c r="C25" s="11">
+        <f>C24*(1-C23)</f>
+        <v/>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>ROYALTY BASE (after co-broke)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Seller share (of company comm)</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Franchise internal split</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Sales director share</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Franchise internal split</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Franchise net share</t>
+        </is>
+      </c>
+      <c r="C28" s="8">
+        <f>1-C26-C27</f>
+        <v/>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Remaining after seller+director</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Franchise net / unit</t>
+        </is>
+      </c>
+      <c r="C29" s="11">
+        <f>C25*C28</f>
+        <v/>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Franchise take-home per local unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Select HQ retained - branded</t>
+        </is>
+      </c>
+      <c r="C30" s="11">
+        <f>C24-C3*C13</f>
+        <v/>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Commission minus branded payout</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
           <t>Select HQ retained - white-label</t>
         </is>
       </c>
-      <c r="C25" s="11">
-        <f>C3*C4-C3*C14</f>
-        <v/>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="C31" s="11">
+        <f>C24-C3*C14</f>
+        <v/>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Commission minus WL payout</t>
         </is>
@@ -1057,11 +1183,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G40"/>
+  <dimension ref="B1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
@@ -1072,7 +1198,7 @@
     <row r="1">
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>DPROPERTY OS - FINANCIAL MODEL v0.6 (blue=headers, grey=totals, yellow=editable)</t>
+          <t>DPROPERTY OS - FINANCIAL MODEL v0.7 (blue=headers, grey=totals, yellow=editable)</t>
         </is>
       </c>
       <c r="C1" s="4" t="n"/>
@@ -1390,27 +1516,27 @@
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>Local royalty + Network &amp; Brand Fund (collected)</t>
+          <t>Local royalty + Fund (on gross-into-company)</t>
         </is>
       </c>
       <c r="C17" s="17">
-        <f>C7*Assumptions!$C$15*Assumptions!$C$16*Assumptions!$C$23*Assumptions!$C$7*C12</f>
+        <f>C7*Assumptions!$C$15*Assumptions!$C$16*Assumptions!$C$25*Assumptions!$C$7*C12</f>
         <v/>
       </c>
       <c r="D17" s="17">
-        <f>D7*Assumptions!$C$15*Assumptions!$C$16*Assumptions!$C$23*Assumptions!$C$7*D12</f>
+        <f>D7*Assumptions!$C$15*Assumptions!$C$16*Assumptions!$C$25*Assumptions!$C$7*D12</f>
         <v/>
       </c>
       <c r="E17" s="17">
-        <f>E7*Assumptions!$C$15*Assumptions!$C$16*Assumptions!$C$23*Assumptions!$C$7*E12</f>
+        <f>E7*Assumptions!$C$15*Assumptions!$C$16*Assumptions!$C$25*Assumptions!$C$7*E12</f>
         <v/>
       </c>
       <c r="F17" s="17">
-        <f>F7*Assumptions!$C$15*Assumptions!$C$16*Assumptions!$C$23*Assumptions!$C$7*F12</f>
+        <f>F7*Assumptions!$C$15*Assumptions!$C$16*Assumptions!$C$25*Assumptions!$C$7*F12</f>
         <v/>
       </c>
       <c r="G17" s="17">
-        <f>G7*Assumptions!$C$15*Assumptions!$C$16*Assumptions!$C$23*Assumptions!$C$7*G12</f>
+        <f>G7*Assumptions!$C$15*Assumptions!$C$16*Assumptions!$C$25*Assumptions!$C$7*G12</f>
         <v/>
       </c>
     </row>
@@ -1421,23 +1547,23 @@
         </is>
       </c>
       <c r="C18" s="17">
-        <f>C7*Assumptions!$C$15*Assumptions!$C$17*Assumptions!$C$24*C12</f>
+        <f>C7*Assumptions!$C$15*Assumptions!$C$17*Assumptions!$C$30*C12</f>
         <v/>
       </c>
       <c r="D18" s="17">
-        <f>D7*Assumptions!$C$15*Assumptions!$C$17*Assumptions!$C$24*D12</f>
+        <f>D7*Assumptions!$C$15*Assumptions!$C$17*Assumptions!$C$30*D12</f>
         <v/>
       </c>
       <c r="E18" s="17">
-        <f>E7*Assumptions!$C$15*Assumptions!$C$17*Assumptions!$C$24*E12</f>
+        <f>E7*Assumptions!$C$15*Assumptions!$C$17*Assumptions!$C$30*E12</f>
         <v/>
       </c>
       <c r="F18" s="17">
-        <f>F7*Assumptions!$C$15*Assumptions!$C$17*Assumptions!$C$24*F12</f>
+        <f>F7*Assumptions!$C$15*Assumptions!$C$17*Assumptions!$C$30*F12</f>
         <v/>
       </c>
       <c r="G18" s="17">
-        <f>G7*Assumptions!$C$15*Assumptions!$C$17*Assumptions!$C$24*G12</f>
+        <f>G7*Assumptions!$C$15*Assumptions!$C$17*Assumptions!$C$30*G12</f>
         <v/>
       </c>
     </row>
@@ -1846,16 +1972,105 @@
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>Founder salary ref: Esteban EUR 4,000/mo (Y1) -&gt; 5,500 (Tranche 2); Miguel EUR 3,000/mo placeholder. Inside 'Salaries'.</t>
-        </is>
-      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>LOCAL DEAL WATERFALL (reference, per unit)</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="n"/>
+      <c r="D39" s="14" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="14" t="n"/>
+      <c r="G39" s="14" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>At 5pct Select commission, branded HQ-retained = franchisee payout = 7,500 per 300k unit. Above 5pct, HQ keeps the upside.</t>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Gross commission (5%)</t>
+        </is>
+      </c>
+      <c r="C40" s="18">
+        <f>Assumptions!$C$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Less external advisors (50%)</t>
+        </is>
+      </c>
+      <c r="C41" s="18">
+        <f>-Assumptions!$C$24*Assumptions!$C$23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Into company (royalty base)</t>
+        </is>
+      </c>
+      <c r="C42" s="19">
+        <f>Assumptions!$C$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Seller (35%)</t>
+        </is>
+      </c>
+      <c r="C43" s="18">
+        <f>-Assumptions!$C$25*Assumptions!$C$26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sales director (10%)</t>
+        </is>
+      </c>
+      <c r="C44" s="18">
+        <f>-Assumptions!$C$25*Assumptions!$C$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Franchise net</t>
+        </is>
+      </c>
+      <c r="C45" s="19">
+        <f>Assumptions!$C$29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>HQ royalty+fund per unit (7.5% of into-company)</t>
+        </is>
+      </c>
+      <c r="C46" s="19">
+        <f>Assumptions!$C$25*Assumptions!$C$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Note: royalty is charged on gross-into-company (2.5%), not franchise net - so agent-comp choices do not change HQ royalty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Founder salary ref: Esteban EUR 4,000/mo -&gt; 5,500 (Tranche 2); Miguel EUR 3,000/mo placeholder. Inside 'Salaries'.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-08-05 21:16:47
</commit_message>
<xml_diff>
--- a/second_brain/09_Exports/Dproperty_OS_Financial_Model.xlsx
+++ b/second_brain/09_Exports/Dproperty_OS_Financial_Model.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B31"/>
+  <dimension ref="B1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -515,26 +515,22 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="B2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>Version: v0.7 (working)   Last built: 2026-07-05   Owner: Esteban</t>
+          <t>Version: v0.8 (working)   Last built: 2026-08-03   Owner: Esteban</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Basis: collected-GCI royalty on GROSS-INTO-COMPANY, 30k/40k staged launch fee, Dproperty Select fixed pct of sale price.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="inlineStr"/>
-    </row>
+          <t>Basis: collected-GCI royalty on GROSS-INTO-COMPANY, 30k/40k staged launch fee, Dproperty Select fixed pct of sale price (branded 2.5pct / white-label 1.5pct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
@@ -570,9 +566,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -601,9 +595,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" t="inlineStr"/>
-    </row>
+    <row r="16"/>
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -625,9 +617,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" t="inlineStr"/>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
@@ -663,9 +653,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" t="inlineStr"/>
-    </row>
+    <row r="26"/>
     <row r="27">
       <c r="B27" s="2" t="inlineStr">
         <is>
@@ -698,6 +686,90 @@
       <c r="B31" t="inlineStr">
         <is>
           <t>4. Minimum royalty floor amount (750/mo placeholder).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>v0.8 CHANGES (2026-08-03) - white-label Select access</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>- White-label Select payout revised 2.0pct -&gt; 1.5pct (external partner broker terms).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>- NEW REVENUE LINE (Model row 19): white-label Dproperty Select, HQ retained.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  v0.7 modelled Select revenue from BRANDED franchises only. White-label had no Select</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  access, so no line existed. The 2026-08-03 decision grants access, so the line is now real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>- HQ keeps 3.5pct of sale price on a white-label Select unit (5pct comm less 1.5pct payout)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  vs 2.5pct on a branded unit (5pct less 2.5pct). HQ earns MORE per white-label Select unit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>- NEW PLACEHOLDER ASSUMPTIONS (C32, C33) - these drive the new line and are UNVALIDATED:</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    white-label units/year = 25 (vs 50 branded); white-label Select mix = 8pct (vs 30pct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Deliberately conservative: white-label carries no investment-only mandate, so most of</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  their volume is assumed to be non-Select. THESE TWO CELLS ARE THE MAIN SENSITIVITY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>5. VALIDATE white-label units/year and Select mix (C32/C33) - highest-leverage open input.</t>
         </is>
       </c>
     </row>
@@ -712,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D31"/>
+  <dimension ref="B1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -903,11 +975,11 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>pct of sale price to partner</t>
+          <t>pct of sale price - EXTERNAL PARTNER BROKER terms (rev 2026-08-03, was 2.0pct)</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1240,37 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Commission minus WL payout</t>
+          <t>Commission minus WL payout -&gt; HQ keeps 3.5pct of price</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>White-label units / year</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER - smaller than branded (50). VALIDATE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>White-label Select mix</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER - WL is not investment-mandated. VALIDATE.</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1198,7 +1300,7 @@
     <row r="1">
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>DPROPERTY OS - FINANCIAL MODEL v0.7 (blue=headers, grey=totals, yellow=editable)</t>
+          <t>DPROPERTY OS - FINANCIAL MODEL v0.8 (blue=headers, grey=totals, yellow=editable)</t>
         </is>
       </c>
       <c r="C1" s="4" t="n"/>
@@ -1570,233 +1672,239 @@
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>White-label setup fees</t>
+          <t>Dproperty Select - white-label HQ retained</t>
         </is>
       </c>
       <c r="C19" s="17">
-        <f>C9*Assumptions!$C$18</f>
+        <f>C10*Assumptions!$C$32*Assumptions!$C$33*Assumptions!$C$31*C12</f>
         <v/>
       </c>
       <c r="D19" s="17">
-        <f>D9*Assumptions!$C$18</f>
+        <f>D10*Assumptions!$C$32*Assumptions!$C$33*Assumptions!$C$31*D12</f>
         <v/>
       </c>
       <c r="E19" s="17">
-        <f>E9*Assumptions!$C$18</f>
+        <f>E10*Assumptions!$C$32*Assumptions!$C$33*Assumptions!$C$31*E12</f>
         <v/>
       </c>
       <c r="F19" s="17">
-        <f>F9*Assumptions!$C$18</f>
+        <f>F10*Assumptions!$C$32*Assumptions!$C$33*Assumptions!$C$31*F12</f>
         <v/>
       </c>
       <c r="G19" s="17">
-        <f>G9*Assumptions!$C$18</f>
+        <f>G10*Assumptions!$C$32*Assumptions!$C$33*Assumptions!$C$31*G12</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>White-label recurring</t>
+          <t>White-label setup fees</t>
         </is>
       </c>
       <c r="C20" s="17">
-        <f>C10*Assumptions!$C$19*12</f>
+        <f>C9*Assumptions!$C$18</f>
         <v/>
       </c>
       <c r="D20" s="17">
-        <f>D10*Assumptions!$C$19*12</f>
+        <f>D9*Assumptions!$C$18</f>
         <v/>
       </c>
       <c r="E20" s="17">
-        <f>E10*Assumptions!$C$19*12</f>
+        <f>E9*Assumptions!$C$18</f>
         <v/>
       </c>
       <c r="F20" s="17">
-        <f>F10*Assumptions!$C$19*12</f>
+        <f>F9*Assumptions!$C$18</f>
         <v/>
       </c>
       <c r="G20" s="17">
-        <f>G10*Assumptions!$C$19*12</f>
+        <f>G9*Assumptions!$C$18</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>GoHighLevel resale margin</t>
+          <t>White-label recurring</t>
         </is>
       </c>
       <c r="C21" s="17">
-        <f>(C7+C10)*Assumptions!$C$20*12</f>
+        <f>C10*Assumptions!$C$19*12</f>
         <v/>
       </c>
       <c r="D21" s="17">
-        <f>(D7+D10)*Assumptions!$C$20*12</f>
+        <f>D10*Assumptions!$C$19*12</f>
         <v/>
       </c>
       <c r="E21" s="17">
-        <f>(E7+E10)*Assumptions!$C$20*12</f>
+        <f>E10*Assumptions!$C$19*12</f>
         <v/>
       </c>
       <c r="F21" s="17">
-        <f>(F7+F10)*Assumptions!$C$20*12</f>
+        <f>F10*Assumptions!$C$19*12</f>
         <v/>
       </c>
       <c r="G21" s="17">
-        <f>(G7+G10)*Assumptions!$C$20*12</f>
+        <f>G10*Assumptions!$C$19*12</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
+          <t>GoHighLevel resale margin</t>
+        </is>
+      </c>
+      <c r="C22" s="17">
+        <f>(C7+C10)*Assumptions!$C$20*12</f>
+        <v/>
+      </c>
+      <c r="D22" s="17">
+        <f>(D7+D10)*Assumptions!$C$20*12</f>
+        <v/>
+      </c>
+      <c r="E22" s="17">
+        <f>(E7+E10)*Assumptions!$C$20*12</f>
+        <v/>
+      </c>
+      <c r="F22" s="17">
+        <f>(F7+F10)*Assumptions!$C$20*12</f>
+        <v/>
+      </c>
+      <c r="G22" s="17">
+        <f>(G7+G10)*Assumptions!$C$20*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
           <t>Developer Sales OS</t>
         </is>
       </c>
-      <c r="C22" s="17">
+      <c r="C23" s="17">
         <f>C11*Assumptions!$C$21</f>
         <v/>
       </c>
-      <c r="D22" s="17">
+      <c r="D23" s="17">
         <f>D11*Assumptions!$C$21</f>
         <v/>
       </c>
-      <c r="E22" s="17">
+      <c r="E23" s="17">
         <f>E11*Assumptions!$C$21</f>
         <v/>
       </c>
-      <c r="F22" s="17">
+      <c r="F23" s="17">
         <f>F11*Assumptions!$C$21</f>
         <v/>
       </c>
-      <c r="G22" s="17">
+      <c r="G23" s="17">
         <f>G11*Assumptions!$C$21</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>TOTAL REVENUE</t>
         </is>
       </c>
-      <c r="C23" s="11">
-        <f>SUM(C15:C22)</f>
-        <v/>
-      </c>
-      <c r="D23" s="11">
-        <f>SUM(D15:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="11">
-        <f>SUM(E15:E22)</f>
-        <v/>
-      </c>
-      <c r="F23" s="11">
-        <f>SUM(F15:F22)</f>
-        <v/>
-      </c>
-      <c r="G23" s="11">
-        <f>SUM(G15:G22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="13" t="inlineStr">
+      <c r="C24" s="11">
+        <f>SUM(C15:C23)</f>
+        <v/>
+      </c>
+      <c r="D24" s="11">
+        <f>SUM(D15:D23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="11">
+        <f>SUM(E15:E23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="11">
+        <f>SUM(F15:F23)</f>
+        <v/>
+      </c>
+      <c r="G24" s="11">
+        <f>SUM(G15:G23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>OPERATING COSTS (USD) - editable planning estimates</t>
         </is>
       </c>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Salaries (founders + team)</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>220000</v>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>300000</v>
-      </c>
-      <c r="F26" s="5" t="n">
-        <v>400000</v>
-      </c>
-      <c r="G26" s="5" t="n">
-        <v>500000</v>
-      </c>
+      <c r="C26" s="14" t="n"/>
+      <c r="D26" s="14" t="n"/>
+      <c r="E26" s="14" t="n"/>
+      <c r="F26" s="14" t="n"/>
+      <c r="G26" s="14" t="n"/>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>Product / technology</t>
+          <t>Salaries (founders + team)</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>80000</v>
+        <v>150000</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>70000</v>
+        <v>220000</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>80000</v>
+        <v>300000</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>90000</v>
+        <v>400000</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>100000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>Legal / compliance</t>
+          <t>Product / technology</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>60000</v>
+        <v>80000</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>40000</v>
+        <v>70000</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>40000</v>
+        <v>90000</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>40000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>Training / content</t>
+          <t>Legal / compliance</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D29" s="5" t="n">
         <v>40000</v>
       </c>
-      <c r="D29" s="5" t="n">
-        <v>30000</v>
-      </c>
       <c r="E29" s="5" t="n">
-        <v>30000</v>
+        <v>40000</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>35000</v>
+        <v>40000</v>
       </c>
       <c r="G29" s="5" t="n">
         <v>40000</v>
@@ -1805,270 +1913,295 @@
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>Customer success / implementation</t>
+          <t>Training / content</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D30" s="5" t="n">
         <v>30000</v>
       </c>
-      <c r="D30" s="5" t="n">
-        <v>50000</v>
-      </c>
       <c r="E30" s="5" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>90000</v>
+        <v>35000</v>
       </c>
       <c r="G30" s="5" t="n">
-        <v>110000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sales / BD / travel</t>
+          <t>Customer success / implementation</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
-        <v>40000</v>
+        <v>30000</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>50000</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>60000</v>
+        <v>70000</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>70000</v>
+        <v>90000</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>80000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>Hosting / tools / admin</t>
+          <t>Sales / BD / travel</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
-        <v>30000</v>
+        <v>40000</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>35000</v>
+        <v>50000</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>55000</v>
+        <v>70000</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>65000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
+          <t>Hosting / tools / admin</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>35000</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>55000</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
           <t>Contingency</t>
         </is>
       </c>
-      <c r="C33" s="5" t="n">
+      <c r="C34" s="5" t="n">
         <v>15000</v>
       </c>
-      <c r="D33" s="5" t="n">
+      <c r="D34" s="5" t="n">
         <v>15000</v>
       </c>
-      <c r="E33" s="5" t="n">
+      <c r="E34" s="5" t="n">
         <v>20000</v>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="F34" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="G33" s="5" t="n">
+      <c r="G34" s="5" t="n">
         <v>30000</v>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="2" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>TOTAL OPEX</t>
         </is>
       </c>
-      <c r="C34" s="11">
-        <f>SUM(C26:C33)</f>
-        <v/>
-      </c>
-      <c r="D34" s="11">
-        <f>SUM(D26:D33)</f>
-        <v/>
-      </c>
-      <c r="E34" s="11">
-        <f>SUM(E26:E33)</f>
-        <v/>
-      </c>
-      <c r="F34" s="11">
-        <f>SUM(F26:F33)</f>
-        <v/>
-      </c>
-      <c r="G34" s="11">
-        <f>SUM(G26:G33)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>EBITDA</t>
-        </is>
-      </c>
-      <c r="C36" s="11">
-        <f>C23-C34</f>
-        <v/>
-      </c>
-      <c r="D36" s="11">
-        <f>D23-D34</f>
-        <v/>
-      </c>
-      <c r="E36" s="11">
-        <f>E23-E34</f>
-        <v/>
-      </c>
-      <c r="F36" s="11">
-        <f>F23-F34</f>
-        <v/>
-      </c>
-      <c r="G36" s="11">
-        <f>G23-G34</f>
-        <v/>
-      </c>
-    </row>
+      <c r="C35" s="11">
+        <f>SUM(C27:C34)</f>
+        <v/>
+      </c>
+      <c r="D35" s="11">
+        <f>SUM(D27:D34)</f>
+        <v/>
+      </c>
+      <c r="E35" s="11">
+        <f>SUM(E27:E34)</f>
+        <v/>
+      </c>
+      <c r="F35" s="11">
+        <f>SUM(F27:F34)</f>
+        <v/>
+      </c>
+      <c r="G35" s="11">
+        <f>SUM(G27:G34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="2" t="inlineStr">
         <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="C37" s="11">
+        <f>C24-C35</f>
+        <v/>
+      </c>
+      <c r="D37" s="11">
+        <f>D24-D35</f>
+        <v/>
+      </c>
+      <c r="E37" s="11">
+        <f>E24-E35</f>
+        <v/>
+      </c>
+      <c r="F37" s="11">
+        <f>F24-F35</f>
+        <v/>
+      </c>
+      <c r="G37" s="11">
+        <f>G24-G35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="2" t="inlineStr">
+        <is>
           <t>EBITDA margin</t>
         </is>
       </c>
-      <c r="C37" s="8">
-        <f>IFERROR(C36/C23,0)</f>
-        <v/>
-      </c>
-      <c r="D37" s="8">
-        <f>IFERROR(D36/D23,0)</f>
-        <v/>
-      </c>
-      <c r="E37" s="8">
-        <f>IFERROR(E36/E23,0)</f>
-        <v/>
-      </c>
-      <c r="F37" s="8">
-        <f>IFERROR(F36/F23,0)</f>
-        <v/>
-      </c>
-      <c r="G37" s="8">
-        <f>IFERROR(G36/G23,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="13" t="inlineStr">
+      <c r="C38" s="8">
+        <f>IFERROR(C37/C24,0)</f>
+        <v/>
+      </c>
+      <c r="D38" s="8">
+        <f>IFERROR(D37/D24,0)</f>
+        <v/>
+      </c>
+      <c r="E38" s="8">
+        <f>IFERROR(E37/E24,0)</f>
+        <v/>
+      </c>
+      <c r="F38" s="8">
+        <f>IFERROR(F37/F24,0)</f>
+        <v/>
+      </c>
+      <c r="G38" s="8">
+        <f>IFERROR(G37/G24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>LOCAL DEAL WATERFALL (reference, per unit)</t>
         </is>
       </c>
-      <c r="C39" s="14" t="n"/>
-      <c r="D39" s="14" t="n"/>
-      <c r="E39" s="14" t="n"/>
-      <c r="F39" s="14" t="n"/>
-      <c r="G39" s="14" t="n"/>
-    </row>
-    <row r="40">
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Gross commission (5%)</t>
-        </is>
-      </c>
-      <c r="C40" s="18">
-        <f>Assumptions!$C$24</f>
-        <v/>
-      </c>
+      <c r="C40" s="14" t="n"/>
+      <c r="D40" s="14" t="n"/>
+      <c r="E40" s="14" t="n"/>
+      <c r="F40" s="14" t="n"/>
+      <c r="G40" s="14" t="n"/>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Less external advisors (50%)</t>
+          <t>Gross commission (5%)</t>
         </is>
       </c>
       <c r="C41" s="18">
-        <f>-Assumptions!$C$24*Assumptions!$C$23</f>
+        <f>Assumptions!$C$24</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>Into company (royalty base)</t>
-        </is>
-      </c>
-      <c r="C42" s="19">
-        <f>Assumptions!$C$25</f>
+          <t xml:space="preserve">  Less external advisors (50%)</t>
+        </is>
+      </c>
+      <c r="C42" s="18">
+        <f>-Assumptions!$C$24*Assumptions!$C$23</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Seller (35%)</t>
-        </is>
-      </c>
-      <c r="C43" s="18">
-        <f>-Assumptions!$C$25*Assumptions!$C$26</f>
+          <t>Into company (royalty base)</t>
+        </is>
+      </c>
+      <c r="C43" s="19">
+        <f>Assumptions!$C$25</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sales director (10%)</t>
+          <t xml:space="preserve">  Seller (35%)</t>
         </is>
       </c>
       <c r="C44" s="18">
-        <f>-Assumptions!$C$25*Assumptions!$C$27</f>
+        <f>-Assumptions!$C$25*Assumptions!$C$26</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>Franchise net</t>
-        </is>
-      </c>
-      <c r="C45" s="19">
-        <f>Assumptions!$C$29</f>
+          <t xml:space="preserve">  Sales director (10%)</t>
+        </is>
+      </c>
+      <c r="C45" s="18">
+        <f>-Assumptions!$C$25*Assumptions!$C$27</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
+          <t>Franchise net</t>
+        </is>
+      </c>
+      <c r="C46" s="19">
+        <f>Assumptions!$C$29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
           <t>HQ royalty+fund per unit (7.5% of into-company)</t>
         </is>
       </c>
-      <c r="C46" s="19">
+      <c r="C47" s="19">
         <f>Assumptions!$C$25*Assumptions!$C$7</f>
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>Note: royalty is charged on gross-into-company (2.5%), not franchise net - so agent-comp choices do not change HQ royalty.</t>
-        </is>
-      </c>
-    </row>
+    <row r="48"/>
     <row r="49">
       <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Note: royalty is charged on gross-into-company (2.5%), not franchise net - so agent-comp choices do not change HQ royalty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>Founder salary ref: Esteban EUR 4,000/mo -&gt; 5,500 (Tranche 2); Miguel EUR 3,000/mo placeholder. Inside 'Salaries'.</t>
         </is>

</xml_diff>